<commit_message>
demo ces: update forms
</commit_message>
<xml_diff>
--- a/Demo/CES/demo_ces_9999_3_cap.xlsx
+++ b/Demo/CES/demo_ces_9999_3_cap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\CES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bonhe\Repositories\dsa-forms\Demo\CES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A08A014-668D-4F89-883B-7A44D4132947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D503D55E-C9E5-4584-BC24-F5EFD4C6D335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{9CE59DC2-AD45-4C3F-AC96-D1E4C9324384}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9CE59DC2-AD45-4C3F-AC96-D1E4C9324384}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="394">
   <si>
     <t>type</t>
   </si>
@@ -326,9 +326,6 @@
     <t>col_3</t>
   </si>
   <si>
-    <t>demo_ces_9999_3_cap</t>
-  </si>
-  <si>
     <t>label::English</t>
   </si>
   <si>
@@ -857,9 +854,6 @@
     <t>${p_site_id}</t>
   </si>
   <si>
-    <t>(Demo) CES - 3. Formulaire KAP</t>
-  </si>
-  <si>
     <t>Which disease does this KAP concern?</t>
   </si>
   <si>
@@ -1203,6 +1197,27 @@
   </si>
   <si>
     <t>sch_prevention_other</t>
+  </si>
+  <si>
+    <t>Do you know anyone in this village who has blood in urine or blood in stool?</t>
+  </si>
+  <si>
+    <t>sch_know_peopl_blood_ur</t>
+  </si>
+  <si>
+    <t>sch_know_symptom</t>
+  </si>
+  <si>
+    <t>sch</t>
+  </si>
+  <si>
+    <t>(Demo) CES - 3. Formulaire KAP V2</t>
+  </si>
+  <si>
+    <t>demo_ces_9999_3_cap_v2</t>
+  </si>
+  <si>
+    <t>selected(${d_disease_list}, 'SCH')</t>
   </si>
 </sst>
 </file>
@@ -1782,7 +1797,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U77"/>
+  <dimension ref="A1:U76"/>
   <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" style="12" bestFit="1" customWidth="1"/>
@@ -1811,16 +1826,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>97</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>98</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>4</v>
@@ -1850,13 +1865,13 @@
         <v>91</v>
       </c>
       <c r="P1" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q1" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="Q1" s="10" t="s">
+      <c r="R1" s="10" t="s">
         <v>101</v>
-      </c>
-      <c r="R1" s="10" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
@@ -1864,10 +1879,10 @@
         <v>77</v>
       </c>
       <c r="B2" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" s="21" t="s">
         <v>104</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>105</v>
       </c>
       <c r="D2" s="21"/>
       <c r="E2" s="22"/>
@@ -1892,10 +1907,10 @@
         <v>24</v>
       </c>
       <c r="B3" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="26" t="s">
         <v>106</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>107</v>
       </c>
       <c r="D3" s="26"/>
       <c r="E3" s="27"/>
@@ -1924,10 +1939,10 @@
         <v>24</v>
       </c>
       <c r="B4" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="26" t="s">
         <v>108</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>109</v>
       </c>
       <c r="D4" s="26"/>
       <c r="E4" s="27"/>
@@ -1944,7 +1959,7 @@
         <v>93</v>
       </c>
       <c r="N4" s="29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O4" s="25"/>
       <c r="P4" s="25"/>
@@ -1958,10 +1973,10 @@
         <v>24</v>
       </c>
       <c r="B5" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>111</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>112</v>
       </c>
       <c r="D5" s="26"/>
       <c r="E5" s="27"/>
@@ -1979,7 +1994,7 @@
       </c>
       <c r="N5" s="24"/>
       <c r="O5" s="29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P5" s="25"/>
       <c r="Q5" s="24"/>
@@ -1992,10 +2007,10 @@
         <v>24</v>
       </c>
       <c r="B6" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="26" t="s">
         <v>114</v>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>115</v>
       </c>
       <c r="D6" s="26"/>
       <c r="E6" s="27"/>
@@ -2009,12 +2024,12 @@
       <c r="K6" s="24"/>
       <c r="L6" s="24"/>
       <c r="M6" s="24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="N6" s="25"/>
       <c r="O6" s="25"/>
       <c r="P6" s="24" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Q6" s="24"/>
       <c r="R6" s="24"/>
@@ -2022,77 +2037,69 @@
       <c r="U6" s="31"/>
     </row>
     <row r="7" spans="1:21" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="37"/>
-      <c r="B7" s="37"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="40"/>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="39"/>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="39"/>
-      <c r="R7" s="39"/>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="D8" s="22"/>
-      <c r="E8" s="34" t="s">
-        <v>74</v>
-      </c>
-      <c r="F8" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="20" t="s">
+      <c r="A7" s="20" t="s">
+        <v>274</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>273</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>272</v>
+      </c>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="N8" s="22"/>
-      <c r="O8" s="29"/>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22" t="s">
-        <v>272</v>
-      </c>
-      <c r="R8" s="22"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="33"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="33"/>
+      <c r="Q7" s="33"/>
+      <c r="R7" s="33"/>
+    </row>
+    <row r="8" spans="1:21" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="37"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
+      <c r="Q8" s="39"/>
+      <c r="R8" s="39"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D9" s="22"/>
       <c r="E9" s="34" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="G9" s="22"/>
       <c r="H9" s="22"/>
@@ -2102,37 +2109,41 @@
       <c r="J9" s="22"/>
       <c r="K9" s="22"/>
       <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
+      <c r="M9" s="33" t="s">
+        <v>270</v>
+      </c>
       <c r="N9" s="22"/>
-      <c r="O9" s="22"/>
+      <c r="O9" s="29"/>
       <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
+      <c r="Q9" s="22" t="s">
+        <v>271</v>
+      </c>
       <c r="R9" s="22"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
+      <c r="E10" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>87</v>
+      </c>
       <c r="G10" s="22"/>
-      <c r="H10" s="22" t="s">
-        <v>270</v>
-      </c>
+      <c r="H10" s="22"/>
       <c r="I10" s="20" t="s">
         <v>23</v>
       </c>
       <c r="J10" s="22"/>
-      <c r="K10" s="22" t="s">
-        <v>23</v>
-      </c>
+      <c r="K10" s="22"/>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
       <c r="N10" s="22"/>
@@ -2143,28 +2154,28 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>58</v>
+        <v>122</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>188</v>
+        <v>119</v>
       </c>
       <c r="D11" s="22"/>
-      <c r="E11" s="22" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="22" t="s">
-        <v>73</v>
-      </c>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
+      <c r="H11" s="22" t="s">
+        <v>269</v>
+      </c>
       <c r="I11" s="20" t="s">
         <v>23</v>
       </c>
       <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
+      <c r="K11" s="22" t="s">
+        <v>23</v>
+      </c>
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
@@ -2175,17 +2186,21 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
-        <v>141</v>
+        <v>9</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>124</v>
+        <v>58</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="E12" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>73</v>
+      </c>
       <c r="G12" s="22"/>
       <c r="H12" s="22"/>
       <c r="I12" s="20" t="s">
@@ -2203,13 +2218,13 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
@@ -2229,63 +2244,57 @@
       <c r="Q13" s="22"/>
       <c r="R13" s="22"/>
     </row>
-    <row r="14" spans="1:21" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
-        <v>9</v>
+        <v>144</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="F14" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="G14" s="20"/>
+        <v>59</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
       <c r="H14" s="22"/>
       <c r="I14" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J14" s="20"/>
-      <c r="K14" s="33"/>
-      <c r="L14" s="33"/>
-      <c r="M14" s="33"/>
-      <c r="N14" s="33"/>
-      <c r="O14" s="33"/>
-      <c r="P14" s="33"/>
-      <c r="Q14" s="33"/>
-      <c r="R14" s="33"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="22"/>
+      <c r="Q14" s="22"/>
+      <c r="R14" s="22"/>
     </row>
     <row r="15" spans="1:21" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D15" s="33"/>
-      <c r="E15" s="20" t="s">
-        <v>80</v>
+      <c r="E15" s="33" t="s">
+        <v>81</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G15" s="33" t="s">
-        <v>79</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="G15" s="20"/>
       <c r="H15" s="22"/>
       <c r="I15" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J15" s="33"/>
+      <c r="J15" s="20"/>
       <c r="K15" s="33"/>
       <c r="L15" s="33"/>
       <c r="M15" s="33"/>
@@ -2296,44 +2305,58 @@
       <c r="R15" s="33"/>
     </row>
     <row r="16" spans="1:21" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="37"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37"/>
-      <c r="K16" s="39"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="39"/>
-      <c r="O16" s="39"/>
-      <c r="P16" s="39"/>
-      <c r="Q16" s="39"/>
-      <c r="R16" s="39"/>
+      <c r="A16" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="D16" s="33"/>
+      <c r="E16" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="G16" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H16" s="22"/>
+      <c r="I16" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+      <c r="P16" s="33"/>
+      <c r="Q16" s="33"/>
+      <c r="R16" s="33"/>
     </row>
     <row r="17" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
-        <v>276</v>
+        <v>9</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>275</v>
+        <v>213</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>274</v>
+        <v>202</v>
       </c>
       <c r="D17" s="33"/>
       <c r="E17" s="33"/>
       <c r="F17" s="33"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="22"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
       <c r="I17" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J17" s="20"/>
+      <c r="J17" s="33"/>
       <c r="K17" s="33"/>
       <c r="L17" s="33"/>
       <c r="M17" s="33"/>
@@ -2344,318 +2367,312 @@
       <c r="R17" s="33"/>
     </row>
     <row r="18" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
-        <v>341</v>
-      </c>
-      <c r="B18" s="37" t="s">
-        <v>342</v>
-      </c>
-      <c r="C18" s="37"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="37" t="s">
-        <v>281</v>
-      </c>
-      <c r="H18" s="39"/>
-      <c r="I18" s="37"/>
-      <c r="J18" s="37"/>
-      <c r="K18" s="39"/>
-      <c r="L18" s="39"/>
-      <c r="M18" s="39"/>
-      <c r="N18" s="39"/>
-      <c r="O18" s="39"/>
-      <c r="P18" s="39"/>
-      <c r="Q18" s="39"/>
-      <c r="R18" s="39"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" s="33"/>
+      <c r="K18" s="33"/>
+      <c r="L18" s="33"/>
+      <c r="M18" s="33"/>
+      <c r="N18" s="33"/>
+      <c r="O18" s="33"/>
+      <c r="P18" s="33"/>
+      <c r="Q18" s="33"/>
+      <c r="R18" s="33"/>
+    </row>
+    <row r="19" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="C19" s="22" t="s">
-        <v>193</v>
-      </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
+        <v>65</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
       <c r="I19" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="22"/>
-      <c r="P19" s="22"/>
-      <c r="Q19" s="22"/>
-      <c r="R19" s="22"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="J19" s="33"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
+      <c r="M19" s="33"/>
+      <c r="N19" s="33"/>
+      <c r="O19" s="33"/>
+      <c r="P19" s="33"/>
+      <c r="Q19" s="33"/>
+      <c r="R19" s="33"/>
+    </row>
+    <row r="20" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
-        <v>147</v>
+        <v>9</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>194</v>
-      </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="H20" s="22"/>
+        <v>216</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="H20" s="33"/>
       <c r="I20" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J20" s="20"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="22"/>
-      <c r="P20" s="22"/>
-      <c r="Q20" s="22"/>
-      <c r="R20" s="22"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="33"/>
+      <c r="P20" s="33"/>
+      <c r="Q20" s="33"/>
+      <c r="R20" s="33"/>
+    </row>
+    <row r="21" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>195</v>
-      </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="H21" s="22"/>
+        <v>66</v>
+      </c>
+      <c r="C21" s="33" t="s">
+        <v>206</v>
+      </c>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
       <c r="I21" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J21" s="20"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="22"/>
-      <c r="P21" s="22"/>
-      <c r="Q21" s="22"/>
-      <c r="R21" s="22"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="33"/>
+      <c r="N21" s="33"/>
+      <c r="O21" s="33"/>
+      <c r="P21" s="33"/>
+      <c r="Q21" s="33"/>
+      <c r="R21" s="33"/>
+    </row>
+    <row r="22" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>196</v>
-      </c>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+        <v>217</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
       <c r="G22" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="H22" s="22"/>
+        <v>227</v>
+      </c>
+      <c r="H22" s="33"/>
       <c r="I22" s="20" t="s">
         <v>23</v>
       </c>
       <c r="J22" s="20"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="22"/>
-      <c r="P22" s="22"/>
-      <c r="Q22" s="22"/>
-      <c r="R22" s="22"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+      <c r="N22" s="33"/>
+      <c r="O22" s="33"/>
+      <c r="P22" s="33"/>
+      <c r="Q22" s="33"/>
+      <c r="R22" s="33"/>
+    </row>
+    <row r="23" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>197</v>
-      </c>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+        <v>219</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>208</v>
+      </c>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
       <c r="G23" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="H23" s="22"/>
+        <v>218</v>
+      </c>
+      <c r="H23" s="33"/>
       <c r="I23" s="20" t="s">
         <v>23</v>
       </c>
       <c r="J23" s="20"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="22"/>
-      <c r="O23" s="22"/>
-      <c r="P23" s="22"/>
-      <c r="Q23" s="22"/>
-      <c r="R23" s="22"/>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="33"/>
+      <c r="N23" s="33"/>
+      <c r="O23" s="33"/>
+      <c r="P23" s="33"/>
+      <c r="Q23" s="33"/>
+      <c r="R23" s="33"/>
+    </row>
+    <row r="24" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>128</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>198</v>
-      </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
+        <v>220</v>
+      </c>
+      <c r="C24" s="33" t="s">
+        <v>209</v>
+      </c>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
       <c r="G24" s="20" t="s">
-        <v>178</v>
-      </c>
-      <c r="H24" s="22"/>
+        <v>229</v>
+      </c>
+      <c r="H24" s="33"/>
       <c r="I24" s="20" t="s">
         <v>23</v>
       </c>
       <c r="J24" s="20"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
-      <c r="N24" s="22"/>
-      <c r="O24" s="22"/>
-      <c r="P24" s="22"/>
-      <c r="Q24" s="22"/>
-      <c r="R24" s="22"/>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="33"/>
+      <c r="N24" s="33"/>
+      <c r="O24" s="33"/>
+      <c r="P24" s="33"/>
+      <c r="Q24" s="33"/>
+      <c r="R24" s="33"/>
+    </row>
+    <row r="25" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C25" s="22" t="s">
-        <v>199</v>
-      </c>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
+        <v>221</v>
+      </c>
+      <c r="C25" s="33" t="s">
+        <v>210</v>
+      </c>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="H25" s="33"/>
       <c r="I25" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="22"/>
-      <c r="O25" s="22"/>
-      <c r="P25" s="22"/>
-      <c r="Q25" s="22"/>
-      <c r="R25" s="22"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="J25" s="20"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="33"/>
+      <c r="N25" s="33"/>
+      <c r="O25" s="33"/>
+      <c r="P25" s="33"/>
+      <c r="Q25" s="33"/>
+      <c r="R25" s="33"/>
+    </row>
+    <row r="26" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="C26" s="22" t="s">
-        <v>200</v>
-      </c>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="20" t="s">
-        <v>187</v>
-      </c>
-      <c r="H26" s="22"/>
-      <c r="I26" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J26" s="20"/>
-      <c r="K26" s="22"/>
-      <c r="L26" s="22"/>
-      <c r="M26" s="22"/>
-      <c r="N26" s="22"/>
-      <c r="O26" s="22"/>
-      <c r="P26" s="22"/>
-      <c r="Q26" s="22"/>
-      <c r="R26" s="22"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>130</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>201</v>
-      </c>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="H27" s="22"/>
-      <c r="I27" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J27" s="20"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="22"/>
-      <c r="Q27" s="22"/>
-      <c r="R27" s="22"/>
+        <v>69</v>
+      </c>
+      <c r="C26" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="33"/>
+      <c r="K26" s="33"/>
+      <c r="L26" s="33"/>
+      <c r="M26" s="33"/>
+      <c r="N26" s="33"/>
+      <c r="O26" s="33"/>
+      <c r="P26" s="33"/>
+      <c r="Q26" s="33"/>
+      <c r="R26" s="33"/>
+    </row>
+    <row r="27" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="37" t="s">
+        <v>339</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>340</v>
+      </c>
+      <c r="C27" s="37"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="37" t="s">
+        <v>279</v>
+      </c>
+      <c r="H27" s="39"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="39"/>
+      <c r="L27" s="39"/>
+      <c r="M27" s="39"/>
+      <c r="N27" s="39"/>
+      <c r="O27" s="39"/>
+      <c r="P27" s="39"/>
+      <c r="Q27" s="39"/>
+      <c r="R27" s="39"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
-        <v>9</v>
+        <v>146</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="22"/>
       <c r="F28" s="22"/>
-      <c r="G28" s="20" t="s">
-        <v>135</v>
-      </c>
+      <c r="G28" s="22"/>
       <c r="H28" s="22"/>
       <c r="I28" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J28" s="20"/>
+      <c r="J28" s="22"/>
       <c r="K28" s="22"/>
       <c r="L28" s="22"/>
       <c r="M28" s="22"/>
@@ -2666,67 +2683,81 @@
       <c r="R28" s="22"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="37" t="s">
-        <v>343</v>
-      </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="37"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="37"/>
-      <c r="J29" s="37"/>
-      <c r="K29" s="39"/>
-      <c r="L29" s="39"/>
-      <c r="M29" s="39"/>
-      <c r="N29" s="39"/>
-      <c r="O29" s="39"/>
-      <c r="P29" s="39"/>
-      <c r="Q29" s="39"/>
-      <c r="R29" s="39"/>
+      <c r="A29" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="H29" s="22"/>
+      <c r="I29" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J29" s="20"/>
+      <c r="K29" s="22"/>
+      <c r="L29" s="22"/>
+      <c r="M29" s="22"/>
+      <c r="N29" s="22"/>
+      <c r="O29" s="22"/>
+      <c r="P29" s="22"/>
+      <c r="Q29" s="22"/>
+      <c r="R29" s="22"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="37" t="s">
-        <v>341</v>
-      </c>
-      <c r="B30" s="37" t="s">
-        <v>344</v>
-      </c>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="37" t="s">
-        <v>345</v>
-      </c>
-      <c r="H30" s="39"/>
-      <c r="I30" s="37"/>
-      <c r="J30" s="37"/>
-      <c r="K30" s="39"/>
-      <c r="L30" s="39"/>
-      <c r="M30" s="39"/>
-      <c r="N30" s="39"/>
-      <c r="O30" s="39"/>
-      <c r="P30" s="39"/>
-      <c r="Q30" s="39"/>
-      <c r="R30" s="39"/>
+      <c r="A30" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="H30" s="22"/>
+      <c r="I30" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J30" s="20"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="22"/>
+      <c r="M30" s="22"/>
+      <c r="N30" s="22"/>
+      <c r="O30" s="22"/>
+      <c r="P30" s="22"/>
+      <c r="Q30" s="22"/>
+      <c r="R30" s="22"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
-        <v>132</v>
+        <v>24</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>338</v>
+        <v>126</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>282</v>
+        <v>195</v>
       </c>
       <c r="D31" s="22"/>
       <c r="E31" s="22"/>
       <c r="F31" s="22"/>
-      <c r="G31" s="20"/>
+      <c r="G31" s="20" t="s">
+        <v>161</v>
+      </c>
       <c r="H31" s="22"/>
       <c r="I31" s="20" t="s">
         <v>23</v>
@@ -2743,18 +2774,20 @@
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
-        <v>147</v>
+        <v>27</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>284</v>
+        <v>63</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>283</v>
+        <v>196</v>
       </c>
       <c r="D32" s="22"/>
       <c r="E32" s="22"/>
       <c r="F32" s="22"/>
-      <c r="G32" s="20"/>
+      <c r="G32" s="20" t="s">
+        <v>133</v>
+      </c>
       <c r="H32" s="22"/>
       <c r="I32" s="20" t="s">
         <v>23</v>
@@ -2771,18 +2804,20 @@
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
-        <v>298</v>
+        <v>24</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>299</v>
+        <v>127</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>285</v>
+        <v>197</v>
       </c>
       <c r="D33" s="22"/>
       <c r="E33" s="22"/>
       <c r="F33" s="22"/>
-      <c r="G33" s="20"/>
+      <c r="G33" s="20" t="s">
+        <v>177</v>
+      </c>
       <c r="H33" s="22"/>
       <c r="I33" s="20" t="s">
         <v>23</v>
@@ -2799,25 +2834,23 @@
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>301</v>
+        <v>64</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>300</v>
+        <v>198</v>
       </c>
       <c r="D34" s="22"/>
       <c r="E34" s="22"/>
       <c r="F34" s="22"/>
-      <c r="G34" s="20" t="s">
-        <v>314</v>
-      </c>
+      <c r="G34" s="22"/>
       <c r="H34" s="22"/>
       <c r="I34" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="J34" s="20"/>
+      <c r="J34" s="22"/>
       <c r="K34" s="22"/>
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
@@ -2829,18 +2862,20 @@
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
-        <v>312</v>
+        <v>24</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>313</v>
+        <v>128</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>317</v>
+        <v>199</v>
       </c>
       <c r="D35" s="22"/>
       <c r="E35" s="22"/>
       <c r="F35" s="22"/>
-      <c r="G35" s="20"/>
+      <c r="G35" s="20" t="s">
+        <v>186</v>
+      </c>
       <c r="H35" s="22"/>
       <c r="I35" s="20" t="s">
         <v>23</v>
@@ -2857,19 +2892,19 @@
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
-        <v>8</v>
+        <v>131</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>315</v>
+        <v>129</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>318</v>
+        <v>200</v>
       </c>
       <c r="D36" s="22"/>
       <c r="E36" s="22"/>
       <c r="F36" s="22"/>
       <c r="G36" s="20" t="s">
-        <v>316</v>
+        <v>133</v>
       </c>
       <c r="H36" s="22"/>
       <c r="I36" s="20" t="s">
@@ -2887,18 +2922,20 @@
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
-        <v>331</v>
+        <v>9</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>332</v>
+        <v>130</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>319</v>
+        <v>201</v>
       </c>
       <c r="D37" s="22"/>
       <c r="E37" s="22"/>
       <c r="F37" s="22"/>
-      <c r="G37" s="20"/>
+      <c r="G37" s="20" t="s">
+        <v>134</v>
+      </c>
       <c r="H37" s="22"/>
       <c r="I37" s="20" t="s">
         <v>23</v>
@@ -2914,72 +2951,62 @@
       <c r="R37" s="22"/>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A38" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B38" s="20" t="s">
-        <v>333</v>
-      </c>
-      <c r="C38" s="22" t="s">
-        <v>335</v>
-      </c>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="20" t="s">
-        <v>334</v>
-      </c>
-      <c r="H38" s="22"/>
-      <c r="I38" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J38" s="20"/>
-      <c r="K38" s="22"/>
-      <c r="L38" s="22"/>
-      <c r="M38" s="22"/>
-      <c r="N38" s="22"/>
-      <c r="O38" s="22"/>
-      <c r="P38" s="22"/>
-      <c r="Q38" s="22"/>
-      <c r="R38" s="22"/>
+      <c r="A38" s="37" t="s">
+        <v>341</v>
+      </c>
+      <c r="B38" s="37"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="39"/>
+      <c r="I38" s="37"/>
+      <c r="J38" s="37"/>
+      <c r="K38" s="39"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="39"/>
+      <c r="N38" s="39"/>
+      <c r="O38" s="39"/>
+      <c r="P38" s="39"/>
+      <c r="Q38" s="39"/>
+      <c r="R38" s="39"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A39" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="B39" s="20" t="s">
-        <v>337</v>
-      </c>
-      <c r="C39" s="22" t="s">
-        <v>336</v>
-      </c>
-      <c r="D39" s="22"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J39" s="20"/>
-      <c r="K39" s="22"/>
-      <c r="L39" s="22"/>
-      <c r="M39" s="22"/>
-      <c r="N39" s="22"/>
-      <c r="O39" s="22"/>
-      <c r="P39" s="22"/>
-      <c r="Q39" s="22"/>
-      <c r="R39" s="22"/>
+      <c r="A39" s="37" t="s">
+        <v>339</v>
+      </c>
+      <c r="B39" s="37" t="s">
+        <v>342</v>
+      </c>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="37" t="s">
+        <v>343</v>
+      </c>
+      <c r="H39" s="39"/>
+      <c r="I39" s="37"/>
+      <c r="J39" s="37"/>
+      <c r="K39" s="39"/>
+      <c r="L39" s="39"/>
+      <c r="M39" s="39"/>
+      <c r="N39" s="39"/>
+      <c r="O39" s="39"/>
+      <c r="P39" s="39"/>
+      <c r="Q39" s="39"/>
+      <c r="R39" s="39"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
-        <v>9</v>
+        <v>131</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>339</v>
+        <v>280</v>
       </c>
       <c r="D40" s="22"/>
       <c r="E40" s="22"/>
@@ -3000,65 +3027,81 @@
       <c r="R40" s="22"/>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A41" s="37" t="s">
-        <v>343</v>
-      </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="39"/>
-      <c r="D41" s="39"/>
-      <c r="E41" s="39"/>
-      <c r="F41" s="39"/>
-      <c r="G41" s="37"/>
-      <c r="H41" s="39"/>
-      <c r="I41" s="37"/>
-      <c r="J41" s="37"/>
-      <c r="K41" s="39"/>
-      <c r="L41" s="39"/>
-      <c r="M41" s="39"/>
-      <c r="N41" s="39"/>
-      <c r="O41" s="39"/>
-      <c r="P41" s="39"/>
-      <c r="Q41" s="39"/>
-      <c r="R41" s="39"/>
+      <c r="A41" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="C41" s="22" t="s">
+        <v>281</v>
+      </c>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J41" s="20"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="22"/>
+      <c r="M41" s="22"/>
+      <c r="N41" s="22"/>
+      <c r="O41" s="22"/>
+      <c r="P41" s="22"/>
+      <c r="Q41" s="22"/>
+      <c r="R41" s="22"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A42" s="37" t="s">
-        <v>341</v>
-      </c>
-      <c r="B42" s="37"/>
-      <c r="C42" s="39"/>
-      <c r="D42" s="39"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="39"/>
-      <c r="G42" s="37"/>
-      <c r="H42" s="39"/>
-      <c r="I42" s="37"/>
-      <c r="J42" s="37"/>
-      <c r="K42" s="39"/>
-      <c r="L42" s="39"/>
-      <c r="M42" s="39"/>
-      <c r="N42" s="39"/>
-      <c r="O42" s="39"/>
-      <c r="P42" s="39"/>
-      <c r="Q42" s="39"/>
-      <c r="R42" s="39"/>
+      <c r="A42" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>283</v>
+      </c>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="20"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J42" s="20"/>
+      <c r="K42" s="22"/>
+      <c r="L42" s="22"/>
+      <c r="M42" s="22"/>
+      <c r="N42" s="22"/>
+      <c r="O42" s="22"/>
+      <c r="P42" s="22"/>
+      <c r="Q42" s="22"/>
+      <c r="R42" s="22"/>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="20" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>347</v>
+        <v>299</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>346</v>
+        <v>298</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="22"/>
       <c r="F43" s="22"/>
-      <c r="G43" s="20"/>
+      <c r="G43" s="20" t="s">
+        <v>312</v>
+      </c>
       <c r="H43" s="22"/>
-      <c r="I43" s="20"/>
+      <c r="I43" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J43" s="20"/>
       <c r="K43" s="22"/>
       <c r="L43" s="22"/>
@@ -3071,20 +3114,22 @@
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="20" t="s">
-        <v>147</v>
+        <v>310</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>349</v>
+        <v>311</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>348</v>
+        <v>315</v>
       </c>
       <c r="D44" s="22"/>
       <c r="E44" s="22"/>
       <c r="F44" s="22"/>
       <c r="G44" s="20"/>
       <c r="H44" s="22"/>
-      <c r="I44" s="20"/>
+      <c r="I44" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J44" s="20"/>
       <c r="K44" s="22"/>
       <c r="L44" s="22"/>
@@ -3097,20 +3142,24 @@
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="20" t="s">
-        <v>362</v>
+        <v>8</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>363</v>
+        <v>313</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>364</v>
+        <v>316</v>
       </c>
       <c r="D45" s="22"/>
       <c r="E45" s="22"/>
       <c r="F45" s="22"/>
-      <c r="G45" s="20"/>
+      <c r="G45" s="20" t="s">
+        <v>314</v>
+      </c>
       <c r="H45" s="22"/>
-      <c r="I45" s="20"/>
+      <c r="I45" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J45" s="20"/>
       <c r="K45" s="22"/>
       <c r="L45" s="22"/>
@@ -3123,22 +3172,22 @@
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="20" t="s">
-        <v>8</v>
+        <v>329</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>366</v>
+        <v>330</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>365</v>
+        <v>317</v>
       </c>
       <c r="D46" s="22"/>
       <c r="E46" s="22"/>
       <c r="F46" s="22"/>
-      <c r="G46" s="20" t="s">
-        <v>376</v>
-      </c>
+      <c r="G46" s="20"/>
       <c r="H46" s="22"/>
-      <c r="I46" s="20"/>
+      <c r="I46" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J46" s="20"/>
       <c r="K46" s="22"/>
       <c r="L46" s="22"/>
@@ -3151,20 +3200,24 @@
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
-        <v>373</v>
+        <v>8</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>372</v>
+        <v>331</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>367</v>
+        <v>333</v>
       </c>
       <c r="D47" s="22"/>
       <c r="E47" s="22"/>
       <c r="F47" s="22"/>
-      <c r="G47" s="20"/>
+      <c r="G47" s="20" t="s">
+        <v>332</v>
+      </c>
       <c r="H47" s="22"/>
-      <c r="I47" s="20"/>
+      <c r="I47" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J47" s="20"/>
       <c r="K47" s="22"/>
       <c r="L47" s="22"/>
@@ -3177,22 +3230,22 @@
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="20" t="s">
-        <v>8</v>
+        <v>131</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>375</v>
+        <v>335</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>374</v>
+        <v>334</v>
       </c>
       <c r="D48" s="22"/>
       <c r="E48" s="22"/>
       <c r="F48" s="22"/>
-      <c r="G48" s="20" t="s">
-        <v>376</v>
-      </c>
+      <c r="G48" s="20"/>
       <c r="H48" s="22"/>
-      <c r="I48" s="20"/>
+      <c r="I48" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J48" s="20"/>
       <c r="K48" s="22"/>
       <c r="L48" s="22"/>
@@ -3205,20 +3258,22 @@
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
-        <v>387</v>
+        <v>9</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>386</v>
+        <v>338</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>377</v>
+        <v>337</v>
       </c>
       <c r="D49" s="22"/>
       <c r="E49" s="22"/>
       <c r="F49" s="22"/>
       <c r="G49" s="20"/>
       <c r="H49" s="22"/>
-      <c r="I49" s="20"/>
+      <c r="I49" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J49" s="20"/>
       <c r="K49" s="22"/>
       <c r="L49" s="22"/>
@@ -3230,63 +3285,71 @@
       <c r="R49" s="22"/>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A50" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B50" s="20" t="s">
-        <v>388</v>
-      </c>
-      <c r="C50" s="22" t="s">
-        <v>335</v>
-      </c>
-      <c r="D50" s="22"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="20" t="s">
-        <v>376</v>
-      </c>
-      <c r="H50" s="22"/>
-      <c r="I50" s="20"/>
-      <c r="J50" s="20"/>
-      <c r="K50" s="22"/>
-      <c r="L50" s="22"/>
-      <c r="M50" s="22"/>
-      <c r="N50" s="22"/>
-      <c r="O50" s="22"/>
-      <c r="P50" s="22"/>
-      <c r="Q50" s="22"/>
-      <c r="R50" s="22"/>
+      <c r="A50" s="37" t="s">
+        <v>341</v>
+      </c>
+      <c r="B50" s="37"/>
+      <c r="C50" s="39"/>
+      <c r="D50" s="39"/>
+      <c r="E50" s="39"/>
+      <c r="F50" s="39"/>
+      <c r="G50" s="37"/>
+      <c r="H50" s="39"/>
+      <c r="I50" s="37"/>
+      <c r="J50" s="37"/>
+      <c r="K50" s="39"/>
+      <c r="L50" s="39"/>
+      <c r="M50" s="39"/>
+      <c r="N50" s="39"/>
+      <c r="O50" s="39"/>
+      <c r="P50" s="39"/>
+      <c r="Q50" s="39"/>
+      <c r="R50" s="39"/>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A51" s="20"/>
-      <c r="B51" s="20"/>
-      <c r="C51" s="22"/>
-      <c r="D51" s="22"/>
-      <c r="E51" s="22"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="20"/>
-      <c r="H51" s="22"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-      <c r="K51" s="22"/>
-      <c r="L51" s="22"/>
-      <c r="M51" s="22"/>
-      <c r="N51" s="22"/>
-      <c r="O51" s="22"/>
-      <c r="P51" s="22"/>
-      <c r="Q51" s="22"/>
-      <c r="R51" s="22"/>
+      <c r="A51" s="37" t="s">
+        <v>339</v>
+      </c>
+      <c r="B51" s="37" t="s">
+        <v>390</v>
+      </c>
+      <c r="C51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="39"/>
+      <c r="G51" s="37" t="s">
+        <v>393</v>
+      </c>
+      <c r="H51" s="39"/>
+      <c r="I51" s="37"/>
+      <c r="J51" s="37"/>
+      <c r="K51" s="39"/>
+      <c r="L51" s="39"/>
+      <c r="M51" s="39"/>
+      <c r="N51" s="39"/>
+      <c r="O51" s="39"/>
+      <c r="P51" s="39"/>
+      <c r="Q51" s="39"/>
+      <c r="R51" s="39"/>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A52" s="20"/>
-      <c r="B52" s="20"/>
-      <c r="C52" s="22"/>
+      <c r="A52" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>345</v>
+      </c>
+      <c r="C52" s="22" t="s">
+        <v>344</v>
+      </c>
       <c r="D52" s="22"/>
       <c r="E52" s="22"/>
       <c r="F52" s="22"/>
       <c r="G52" s="20"/>
       <c r="H52" s="22"/>
-      <c r="I52" s="20"/>
+      <c r="I52" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J52" s="20"/>
       <c r="K52" s="22"/>
       <c r="L52" s="22"/>
@@ -3298,15 +3361,23 @@
       <c r="R52" s="22"/>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A53" s="20"/>
-      <c r="B53" s="20"/>
-      <c r="C53" s="22"/>
+      <c r="A53" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>347</v>
+      </c>
+      <c r="C53" s="22" t="s">
+        <v>346</v>
+      </c>
       <c r="D53" s="22"/>
       <c r="E53" s="22"/>
       <c r="F53" s="22"/>
       <c r="G53" s="20"/>
       <c r="H53" s="22"/>
-      <c r="I53" s="20"/>
+      <c r="I53" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J53" s="20"/>
       <c r="K53" s="22"/>
       <c r="L53" s="22"/>
@@ -3318,15 +3389,23 @@
       <c r="R53" s="22"/>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A54" s="20"/>
-      <c r="B54" s="20"/>
-      <c r="C54" s="22"/>
+      <c r="A54" s="20" t="s">
+        <v>360</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>361</v>
+      </c>
+      <c r="C54" s="22" t="s">
+        <v>362</v>
+      </c>
       <c r="D54" s="22"/>
       <c r="E54" s="22"/>
       <c r="F54" s="22"/>
       <c r="G54" s="20"/>
       <c r="H54" s="22"/>
-      <c r="I54" s="20"/>
+      <c r="I54" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J54" s="20"/>
       <c r="K54" s="22"/>
       <c r="L54" s="22"/>
@@ -3338,15 +3417,25 @@
       <c r="R54" s="22"/>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A55" s="20"/>
-      <c r="B55" s="20"/>
-      <c r="C55" s="22"/>
+      <c r="A55" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>364</v>
+      </c>
+      <c r="C55" s="22" t="s">
+        <v>363</v>
+      </c>
       <c r="D55" s="22"/>
       <c r="E55" s="22"/>
       <c r="F55" s="22"/>
-      <c r="G55" s="20"/>
+      <c r="G55" s="20" t="s">
+        <v>374</v>
+      </c>
       <c r="H55" s="22"/>
-      <c r="I55" s="20"/>
+      <c r="I55" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J55" s="20"/>
       <c r="K55" s="22"/>
       <c r="L55" s="22"/>
@@ -3358,15 +3447,23 @@
       <c r="R55" s="22"/>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A56" s="20"/>
-      <c r="B56" s="20"/>
-      <c r="C56" s="22"/>
+      <c r="A56" s="20" t="s">
+        <v>371</v>
+      </c>
+      <c r="B56" s="20" t="s">
+        <v>370</v>
+      </c>
+      <c r="C56" s="22" t="s">
+        <v>365</v>
+      </c>
       <c r="D56" s="22"/>
       <c r="E56" s="22"/>
       <c r="F56" s="22"/>
       <c r="G56" s="20"/>
       <c r="H56" s="22"/>
-      <c r="I56" s="20"/>
+      <c r="I56" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J56" s="20"/>
       <c r="K56" s="22"/>
       <c r="L56" s="22"/>
@@ -3378,15 +3475,25 @@
       <c r="R56" s="22"/>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A57" s="20"/>
-      <c r="B57" s="20"/>
-      <c r="C57" s="22"/>
+      <c r="A57" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B57" s="20" t="s">
+        <v>373</v>
+      </c>
+      <c r="C57" s="22" t="s">
+        <v>372</v>
+      </c>
       <c r="D57" s="22"/>
       <c r="E57" s="22"/>
       <c r="F57" s="22"/>
-      <c r="G57" s="20"/>
+      <c r="G57" s="20" t="s">
+        <v>374</v>
+      </c>
       <c r="H57" s="22"/>
-      <c r="I57" s="20"/>
+      <c r="I57" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J57" s="20"/>
       <c r="K57" s="22"/>
       <c r="L57" s="22"/>
@@ -3398,15 +3505,23 @@
       <c r="R57" s="22"/>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A58" s="20"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="22"/>
+      <c r="A58" s="20" t="s">
+        <v>385</v>
+      </c>
+      <c r="B58" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="C58" s="22" t="s">
+        <v>375</v>
+      </c>
       <c r="D58" s="22"/>
       <c r="E58" s="22"/>
       <c r="F58" s="22"/>
       <c r="G58" s="20"/>
       <c r="H58" s="22"/>
-      <c r="I58" s="20"/>
+      <c r="I58" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J58" s="20"/>
       <c r="K58" s="22"/>
       <c r="L58" s="22"/>
@@ -3418,15 +3533,25 @@
       <c r="R58" s="22"/>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A59" s="20"/>
-      <c r="B59" s="20"/>
-      <c r="C59" s="22"/>
+      <c r="A59" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B59" s="20" t="s">
+        <v>386</v>
+      </c>
+      <c r="C59" s="22" t="s">
+        <v>333</v>
+      </c>
       <c r="D59" s="22"/>
       <c r="E59" s="22"/>
       <c r="F59" s="22"/>
-      <c r="G59" s="20"/>
+      <c r="G59" s="20" t="s">
+        <v>374</v>
+      </c>
       <c r="H59" s="22"/>
-      <c r="I59" s="20"/>
+      <c r="I59" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J59" s="20"/>
       <c r="K59" s="22"/>
       <c r="L59" s="22"/>
@@ -3438,15 +3563,23 @@
       <c r="R59" s="22"/>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A60" s="20"/>
-      <c r="B60" s="20"/>
-      <c r="C60" s="22"/>
+      <c r="A60" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="B60" s="20" t="s">
+        <v>388</v>
+      </c>
+      <c r="C60" s="22" t="s">
+        <v>387</v>
+      </c>
       <c r="D60" s="22"/>
       <c r="E60" s="22"/>
       <c r="F60" s="22"/>
       <c r="G60" s="20"/>
       <c r="H60" s="22"/>
-      <c r="I60" s="20"/>
+      <c r="I60" s="20" t="s">
+        <v>23</v>
+      </c>
       <c r="J60" s="20"/>
       <c r="K60" s="22"/>
       <c r="L60" s="22"/>
@@ -3458,16 +3591,24 @@
       <c r="R60" s="22"/>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A61" s="20"/>
-      <c r="B61" s="20"/>
-      <c r="C61" s="22"/>
+      <c r="A61" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B61" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="C61" s="22" t="s">
+        <v>337</v>
+      </c>
       <c r="D61" s="22"/>
       <c r="E61" s="22"/>
       <c r="F61" s="22"/>
-      <c r="G61" s="22"/>
+      <c r="G61" s="20"/>
       <c r="H61" s="22"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="22"/>
+      <c r="I61" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J61" s="20"/>
       <c r="K61" s="22"/>
       <c r="L61" s="22"/>
       <c r="M61" s="22"/>
@@ -3477,288 +3618,210 @@
       <c r="Q61" s="22"/>
       <c r="R61" s="22"/>
     </row>
-    <row r="62" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B62" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="C62" s="20" t="s">
-        <v>203</v>
-      </c>
-      <c r="D62" s="33"/>
-      <c r="E62" s="33"/>
-      <c r="F62" s="33"/>
-      <c r="G62" s="33"/>
-      <c r="H62" s="33"/>
-      <c r="I62" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J62" s="33"/>
-      <c r="K62" s="33"/>
-      <c r="L62" s="33"/>
-      <c r="M62" s="33"/>
-      <c r="N62" s="33"/>
-      <c r="O62" s="33"/>
-      <c r="P62" s="33"/>
-      <c r="Q62" s="33"/>
-      <c r="R62" s="33"/>
-    </row>
-    <row r="63" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B63" s="20" t="s">
-        <v>216</v>
-      </c>
-      <c r="C63" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="D63" s="33"/>
-      <c r="E63" s="33" t="s">
-        <v>215</v>
-      </c>
-      <c r="F63" s="33"/>
-      <c r="G63" s="33"/>
-      <c r="H63" s="33"/>
-      <c r="I63" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J63" s="33"/>
-      <c r="K63" s="33"/>
-      <c r="L63" s="33"/>
-      <c r="M63" s="33"/>
-      <c r="N63" s="33"/>
-      <c r="O63" s="33"/>
-      <c r="P63" s="33"/>
-      <c r="Q63" s="33"/>
-      <c r="R63" s="33"/>
-    </row>
-    <row r="64" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="20" t="s">
-        <v>147</v>
-      </c>
-      <c r="B64" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C64" s="20" t="s">
-        <v>205</v>
-      </c>
-      <c r="D64" s="33"/>
-      <c r="E64" s="33"/>
-      <c r="F64" s="33"/>
-      <c r="G64" s="33"/>
-      <c r="H64" s="33"/>
-      <c r="I64" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J64" s="33"/>
-      <c r="K64" s="33"/>
-      <c r="L64" s="33"/>
-      <c r="M64" s="33"/>
-      <c r="N64" s="33"/>
-      <c r="O64" s="33"/>
-      <c r="P64" s="33"/>
-      <c r="Q64" s="33"/>
-      <c r="R64" s="33"/>
-    </row>
-    <row r="65" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B65" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="C65" s="20" t="s">
-        <v>206</v>
-      </c>
-      <c r="D65" s="33"/>
-      <c r="E65" s="33"/>
-      <c r="F65" s="33"/>
-      <c r="G65" s="33" t="s">
-        <v>136</v>
-      </c>
-      <c r="H65" s="33"/>
-      <c r="I65" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J65" s="33"/>
-      <c r="K65" s="33"/>
-      <c r="L65" s="33"/>
-      <c r="M65" s="33"/>
-      <c r="N65" s="33"/>
-      <c r="O65" s="33"/>
-      <c r="P65" s="33"/>
-      <c r="Q65" s="33"/>
-      <c r="R65" s="33"/>
-    </row>
-    <row r="66" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="B66" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="C66" s="33" t="s">
-        <v>207</v>
-      </c>
-      <c r="D66" s="33"/>
-      <c r="E66" s="33"/>
-      <c r="F66" s="33"/>
-      <c r="G66" s="33"/>
-      <c r="H66" s="33"/>
-      <c r="I66" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J66" s="33"/>
-      <c r="K66" s="33"/>
-      <c r="L66" s="33"/>
-      <c r="M66" s="33"/>
-      <c r="N66" s="33"/>
-      <c r="O66" s="33"/>
-      <c r="P66" s="33"/>
-      <c r="Q66" s="33"/>
-      <c r="R66" s="33"/>
-    </row>
-    <row r="67" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="B67" s="20" t="s">
-        <v>218</v>
-      </c>
-      <c r="C67" s="33" t="s">
-        <v>208</v>
-      </c>
-      <c r="D67" s="33"/>
-      <c r="E67" s="33"/>
-      <c r="F67" s="33"/>
-      <c r="G67" s="20" t="s">
-        <v>228</v>
-      </c>
-      <c r="H67" s="33"/>
-      <c r="I67" s="20" t="s">
-        <v>23</v>
-      </c>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A62" s="37" t="s">
+        <v>341</v>
+      </c>
+      <c r="B62" s="37"/>
+      <c r="C62" s="39"/>
+      <c r="D62" s="39"/>
+      <c r="E62" s="39"/>
+      <c r="F62" s="39"/>
+      <c r="G62" s="37"/>
+      <c r="H62" s="39"/>
+      <c r="I62" s="37"/>
+      <c r="J62" s="37"/>
+      <c r="K62" s="39"/>
+      <c r="L62" s="39"/>
+      <c r="M62" s="39"/>
+      <c r="N62" s="39"/>
+      <c r="O62" s="39"/>
+      <c r="P62" s="39"/>
+      <c r="Q62" s="39"/>
+      <c r="R62" s="39"/>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A63" s="20"/>
+      <c r="B63" s="20"/>
+      <c r="C63" s="22"/>
+      <c r="D63" s="22"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="20"/>
+      <c r="H63" s="22"/>
+      <c r="I63" s="20"/>
+      <c r="J63" s="20"/>
+      <c r="K63" s="22"/>
+      <c r="L63" s="22"/>
+      <c r="M63" s="22"/>
+      <c r="N63" s="22"/>
+      <c r="O63" s="22"/>
+      <c r="P63" s="22"/>
+      <c r="Q63" s="22"/>
+      <c r="R63" s="22"/>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A64" s="20"/>
+      <c r="B64" s="20"/>
+      <c r="C64" s="22"/>
+      <c r="D64" s="22"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="20"/>
+      <c r="H64" s="22"/>
+      <c r="I64" s="20"/>
+      <c r="J64" s="20"/>
+      <c r="K64" s="22"/>
+      <c r="L64" s="22"/>
+      <c r="M64" s="22"/>
+      <c r="N64" s="22"/>
+      <c r="O64" s="22"/>
+      <c r="P64" s="22"/>
+      <c r="Q64" s="22"/>
+      <c r="R64" s="22"/>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A65" s="20"/>
+      <c r="B65" s="20"/>
+      <c r="C65" s="22"/>
+      <c r="D65" s="22"/>
+      <c r="E65" s="22"/>
+      <c r="F65" s="22"/>
+      <c r="G65" s="20"/>
+      <c r="H65" s="22"/>
+      <c r="I65" s="20"/>
+      <c r="J65" s="20"/>
+      <c r="K65" s="22"/>
+      <c r="L65" s="22"/>
+      <c r="M65" s="22"/>
+      <c r="N65" s="22"/>
+      <c r="O65" s="22"/>
+      <c r="P65" s="22"/>
+      <c r="Q65" s="22"/>
+      <c r="R65" s="22"/>
+    </row>
+    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A66" s="20"/>
+      <c r="B66" s="20"/>
+      <c r="C66" s="22"/>
+      <c r="D66" s="22"/>
+      <c r="E66" s="22"/>
+      <c r="F66" s="22"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="22"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="22"/>
+      <c r="L66" s="22"/>
+      <c r="M66" s="22"/>
+      <c r="N66" s="22"/>
+      <c r="O66" s="22"/>
+      <c r="P66" s="22"/>
+      <c r="Q66" s="22"/>
+      <c r="R66" s="22"/>
+    </row>
+    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A67" s="20"/>
+      <c r="B67" s="20"/>
+      <c r="C67" s="22"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
+      <c r="F67" s="22"/>
+      <c r="G67" s="20"/>
+      <c r="H67" s="22"/>
+      <c r="I67" s="20"/>
       <c r="J67" s="20"/>
-      <c r="K67" s="33"/>
-      <c r="L67" s="33"/>
-      <c r="M67" s="33"/>
-      <c r="N67" s="33"/>
-      <c r="O67" s="33"/>
-      <c r="P67" s="33"/>
-      <c r="Q67" s="33"/>
-      <c r="R67" s="33"/>
-    </row>
-    <row r="68" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B68" s="20" t="s">
-        <v>220</v>
-      </c>
-      <c r="C68" s="33" t="s">
-        <v>209</v>
-      </c>
-      <c r="D68" s="33"/>
-      <c r="E68" s="33"/>
-      <c r="F68" s="33"/>
-      <c r="G68" s="20" t="s">
-        <v>219</v>
-      </c>
-      <c r="H68" s="33"/>
-      <c r="I68" s="20" t="s">
-        <v>23</v>
-      </c>
+      <c r="K67" s="22"/>
+      <c r="L67" s="22"/>
+      <c r="M67" s="22"/>
+      <c r="N67" s="22"/>
+      <c r="O67" s="22"/>
+      <c r="P67" s="22"/>
+      <c r="Q67" s="22"/>
+      <c r="R67" s="22"/>
+    </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A68" s="20"/>
+      <c r="B68" s="20"/>
+      <c r="C68" s="22"/>
+      <c r="D68" s="22"/>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
+      <c r="G68" s="20"/>
+      <c r="H68" s="22"/>
+      <c r="I68" s="20"/>
       <c r="J68" s="20"/>
-      <c r="K68" s="33"/>
-      <c r="L68" s="33"/>
-      <c r="M68" s="33"/>
-      <c r="N68" s="33"/>
-      <c r="O68" s="33"/>
-      <c r="P68" s="33"/>
-      <c r="Q68" s="33"/>
-      <c r="R68" s="33"/>
-    </row>
-    <row r="69" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B69" s="20" t="s">
-        <v>221</v>
-      </c>
-      <c r="C69" s="33" t="s">
-        <v>210</v>
-      </c>
-      <c r="D69" s="33"/>
-      <c r="E69" s="33"/>
-      <c r="F69" s="33"/>
-      <c r="G69" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="H69" s="33"/>
-      <c r="I69" s="20" t="s">
-        <v>23</v>
-      </c>
+      <c r="K68" s="22"/>
+      <c r="L68" s="22"/>
+      <c r="M68" s="22"/>
+      <c r="N68" s="22"/>
+      <c r="O68" s="22"/>
+      <c r="P68" s="22"/>
+      <c r="Q68" s="22"/>
+      <c r="R68" s="22"/>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A69" s="20"/>
+      <c r="B69" s="20"/>
+      <c r="C69" s="22"/>
+      <c r="D69" s="22"/>
+      <c r="E69" s="22"/>
+      <c r="F69" s="22"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="22"/>
+      <c r="I69" s="20"/>
       <c r="J69" s="20"/>
-      <c r="K69" s="33"/>
-      <c r="L69" s="33"/>
-      <c r="M69" s="33"/>
-      <c r="N69" s="33"/>
-      <c r="O69" s="33"/>
-      <c r="P69" s="33"/>
-      <c r="Q69" s="33"/>
-      <c r="R69" s="33"/>
-    </row>
-    <row r="70" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B70" s="20" t="s">
-        <v>222</v>
-      </c>
-      <c r="C70" s="33" t="s">
-        <v>211</v>
-      </c>
-      <c r="D70" s="33"/>
-      <c r="E70" s="33"/>
-      <c r="F70" s="33"/>
-      <c r="G70" s="20" t="s">
-        <v>268</v>
-      </c>
-      <c r="H70" s="33"/>
-      <c r="I70" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J70" s="20"/>
-      <c r="K70" s="33"/>
-      <c r="L70" s="33"/>
-      <c r="M70" s="33"/>
-      <c r="N70" s="33"/>
-      <c r="O70" s="33"/>
-      <c r="P70" s="33"/>
-      <c r="Q70" s="33"/>
-      <c r="R70" s="33"/>
+      <c r="K69" s="22"/>
+      <c r="L69" s="22"/>
+      <c r="M69" s="22"/>
+      <c r="N69" s="22"/>
+      <c r="O69" s="22"/>
+      <c r="P69" s="22"/>
+      <c r="Q69" s="22"/>
+      <c r="R69" s="22"/>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A70" s="20"/>
+      <c r="B70" s="20"/>
+      <c r="C70" s="22"/>
+      <c r="D70" s="22"/>
+      <c r="E70" s="22"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="22"/>
+      <c r="H70" s="22"/>
+      <c r="I70" s="20"/>
+      <c r="J70" s="22"/>
+      <c r="K70" s="22"/>
+      <c r="L70" s="22"/>
+      <c r="M70" s="22"/>
+      <c r="N70" s="22"/>
+      <c r="O70" s="22"/>
+      <c r="P70" s="22"/>
+      <c r="Q70" s="22"/>
+      <c r="R70" s="22"/>
     </row>
     <row r="71" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="20" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B71" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="C71" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="C71" s="20" t="s">
         <v>212</v>
       </c>
       <c r="D71" s="33"/>
-      <c r="E71" s="33"/>
-      <c r="F71" s="33"/>
-      <c r="G71" s="33"/>
-      <c r="H71" s="33"/>
-      <c r="I71" s="20"/>
-      <c r="J71" s="33"/>
-      <c r="K71" s="33"/>
+      <c r="E71" s="35"/>
+      <c r="F71" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="G71" s="35"/>
+      <c r="H71" s="35"/>
+      <c r="I71" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="J71" s="35"/>
+      <c r="K71" s="36"/>
       <c r="L71" s="33"/>
       <c r="M71" s="33"/>
       <c r="N71" s="33"/>
@@ -3767,46 +3830,38 @@
       <c r="Q71" s="33"/>
       <c r="R71" s="33"/>
     </row>
-    <row r="72" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A72" s="20" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>68</v>
-      </c>
-      <c r="C72" s="20" t="s">
-        <v>213</v>
-      </c>
-      <c r="D72" s="33"/>
-      <c r="E72" s="35"/>
-      <c r="F72" s="20" t="s">
-        <v>269</v>
-      </c>
-      <c r="G72" s="35"/>
-      <c r="H72" s="35"/>
-      <c r="I72" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J72" s="35"/>
-      <c r="K72" s="36"/>
-      <c r="L72" s="33"/>
-      <c r="M72" s="33"/>
-      <c r="N72" s="33"/>
-      <c r="O72" s="33"/>
-      <c r="P72" s="33"/>
-      <c r="Q72" s="33"/>
-      <c r="R72" s="33"/>
+        <v>67</v>
+      </c>
+      <c r="C72" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="D72" s="22"/>
+      <c r="E72" s="22"/>
+      <c r="F72" s="22"/>
+      <c r="G72" s="22"/>
+      <c r="H72" s="22"/>
+      <c r="I72" s="20"/>
+      <c r="J72" s="22"/>
+      <c r="K72" s="22"/>
+      <c r="L72" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="M72" s="22"/>
+      <c r="N72" s="22"/>
+      <c r="O72" s="22"/>
+      <c r="P72" s="22"/>
+      <c r="Q72" s="22"/>
+      <c r="R72" s="22"/>
     </row>
     <row r="73" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A73" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B73" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C73" s="22" t="s">
-        <v>94</v>
-      </c>
+      <c r="A73" s="20"/>
+      <c r="B73" s="20"/>
+      <c r="C73" s="22"/>
       <c r="D73" s="22"/>
       <c r="E73" s="22"/>
       <c r="F73" s="22"/>
@@ -3815,9 +3870,7 @@
       <c r="I73" s="20"/>
       <c r="J73" s="22"/>
       <c r="K73" s="22"/>
-      <c r="L73" s="22" t="s">
-        <v>8</v>
-      </c>
+      <c r="L73" s="22"/>
       <c r="M73" s="22"/>
       <c r="N73" s="22"/>
       <c r="O73" s="22"/>
@@ -3826,15 +3879,19 @@
       <c r="R73" s="22"/>
     </row>
     <row r="74" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A74" s="20"/>
-      <c r="B74" s="20"/>
+      <c r="A74" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B74" s="20" t="s">
+        <v>70</v>
+      </c>
       <c r="C74" s="22"/>
       <c r="D74" s="22"/>
       <c r="E74" s="22"/>
       <c r="F74" s="22"/>
       <c r="G74" s="22"/>
       <c r="H74" s="22"/>
-      <c r="I74" s="20"/>
+      <c r="I74" s="22"/>
       <c r="J74" s="22"/>
       <c r="K74" s="22"/>
       <c r="L74" s="22"/>
@@ -3847,10 +3904,10 @@
     </row>
     <row r="75" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A75" s="20" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B75" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C75" s="22"/>
       <c r="D75" s="22"/>
@@ -3870,31 +3927,7 @@
       <c r="R75" s="22"/>
     </row>
     <row r="76" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A76" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B76" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="C76" s="22"/>
-      <c r="D76" s="22"/>
-      <c r="E76" s="22"/>
-      <c r="F76" s="22"/>
-      <c r="G76" s="22"/>
-      <c r="H76" s="22"/>
-      <c r="I76" s="22"/>
-      <c r="J76" s="22"/>
-      <c r="K76" s="22"/>
-      <c r="L76" s="22"/>
-      <c r="M76" s="22"/>
-      <c r="N76" s="22"/>
-      <c r="O76" s="22"/>
-      <c r="P76" s="22"/>
-      <c r="Q76" s="22"/>
-      <c r="R76" s="22"/>
-    </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="C77" s="13"/>
+      <c r="C76" s="13"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1"/>
@@ -3931,7 +3964,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D1" s="16" t="s">
         <v>84</v>
@@ -4002,57 +4035,57 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B11" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>137</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B12" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C12" s="14" t="s">
         <v>139</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>149</v>
-      </c>
       <c r="C13" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -4061,79 +4094,79 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="B15" s="14" t="s">
-        <v>143</v>
-      </c>
       <c r="C15" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -4141,10 +4174,10 @@
         <v>26</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -4152,10 +4185,10 @@
         <v>26</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -4163,10 +4196,10 @@
         <v>26</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -4174,10 +4207,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -4185,10 +4218,10 @@
         <v>26</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -4196,10 +4229,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -4207,10 +4240,10 @@
         <v>26</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -4218,10 +4251,10 @@
         <v>26</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -4229,10 +4262,10 @@
         <v>28</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -4240,10 +4273,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -4251,10 +4284,10 @@
         <v>28</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -4262,10 +4295,10 @@
         <v>28</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -4273,10 +4306,10 @@
         <v>28</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -4284,10 +4317,10 @@
         <v>30</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -4295,10 +4328,10 @@
         <v>30</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -4306,10 +4339,10 @@
         <v>30</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -4317,10 +4350,10 @@
         <v>30</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -4328,10 +4361,10 @@
         <v>30</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -4339,10 +4372,10 @@
         <v>30</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -4350,10 +4383,10 @@
         <v>52</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -4361,10 +4394,10 @@
         <v>52</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -4372,10 +4405,10 @@
         <v>52</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -4383,10 +4416,10 @@
         <v>52</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -4394,10 +4427,10 @@
         <v>55</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -4405,10 +4438,10 @@
         <v>55</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -4416,10 +4449,10 @@
         <v>55</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -4427,10 +4460,10 @@
         <v>55</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -4438,10 +4471,10 @@
         <v>55</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -4449,10 +4482,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -4460,10 +4493,10 @@
         <v>55</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -4471,10 +4504,10 @@
         <v>55</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -4482,10 +4515,10 @@
         <v>55</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
@@ -4493,10 +4526,10 @@
         <v>56</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
@@ -4504,10 +4537,10 @@
         <v>56</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -4515,10 +4548,10 @@
         <v>56</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -4526,10 +4559,10 @@
         <v>56</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
@@ -4537,10 +4570,10 @@
         <v>56</v>
       </c>
       <c r="B65" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -4548,10 +4581,10 @@
         <v>56</v>
       </c>
       <c r="B66" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -4559,10 +4592,10 @@
         <v>56</v>
       </c>
       <c r="B67" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
@@ -4570,10 +4603,10 @@
         <v>56</v>
       </c>
       <c r="B68" s="14" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -4581,10 +4614,10 @@
         <v>56</v>
       </c>
       <c r="B69" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -4592,527 +4625,527 @@
         <v>56</v>
       </c>
       <c r="B70" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B72" s="14" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="B73" s="14" t="s">
         <v>277</v>
       </c>
-      <c r="B73" s="14" t="s">
-        <v>279</v>
-      </c>
       <c r="C73" s="14" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B74" s="14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B76" s="14" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B81" s="14" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B82" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B83" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B85" s="14" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B86" s="14" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C86" s="14" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B87" s="14" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C87" s="14" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B88" s="14" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B89" s="14" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C89" s="14" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B90" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C90" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B93" s="14" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B94" s="14" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B95" s="14" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B96" s="14" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C96" s="14" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B97" s="14" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B98" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C98" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="14" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B99" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C99" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B101" s="14" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B102" s="14" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C102" s="14" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B103" s="14" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C103" s="14" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B104" s="14" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C104" s="14" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B105" s="14" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C105" s="14" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B106" s="14" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C106" s="14" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B107" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C107" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="14" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B108" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C108" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B110" s="14" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C110" s="14" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B111" s="14" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C111" s="14" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B112" s="14" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C112" s="14" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B113" s="14" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C113" s="14" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B114" s="14" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C114" s="14" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B115" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C115" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B116" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C116" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B118" s="14" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C118" s="14" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B119" s="14" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C119" s="14" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B120" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C120" s="14" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B121" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C121" s="14" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B122" s="14" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C122" s="14" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B123" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C123" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B124" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C124" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -5153,13 +5186,13 @@
     </row>
     <row r="2" spans="1:3" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>273</v>
+        <v>391</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>96</v>
+        <v>392</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -5232,24 +5265,24 @@
     </row>
     <row r="37" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="39" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>